<commit_message>
Pequeñas ediciones a cuadernos y diccionarios de datos; agregando readme en inglés
</commit_message>
<xml_diff>
--- a/para_figuras/para_mapa_interactivo/tabla_estaciones_migratorias.xlsx
+++ b/para_figuras/para_mapa_interactivo/tabla_estaciones_migratorias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C105"/>
+  <dimension ref="A1:C155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,99 +461,87 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>10007</t>
-        </is>
+      <c r="A3" s="1" t="n">
+        <v>28032</v>
       </c>
       <c r="B3" t="n">
         <v>1</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>Reynosa</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>10007</v>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>Gómez Palacio</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>20067</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C4" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="1" t="n">
+        <v>20067</v>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="inlineStr">
         <is>
           <t>Oaxaca de Juárez</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>20067</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C5" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="1" t="n">
+        <v>20067</v>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="inlineStr">
         <is>
           <t>Oaxaca de Juárez</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>28038</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>1</v>
-      </c>
-      <c r="C6" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="1" t="n">
+        <v>10007</v>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Gómez Palacio</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>28038</v>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" t="inlineStr">
         <is>
           <t>Tampico</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>28038</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Tampico</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>19026</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Guadalupe</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>19026</t>
+          <t>28038</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -561,44 +549,42 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Guadalupe</t>
+          <t>Tampico</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>10007</t>
+          <t>19026</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Gómez Palacio</t>
+          <t>Guadalupe</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>30193</t>
-        </is>
+      <c r="A11" s="1" t="n">
+        <v>28038</v>
       </c>
       <c r="B11" t="n">
         <v>1</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Veracruz</t>
+          <t>Tampico</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>30193</t>
+          <t>28032</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -606,15 +592,13 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Veracruz</t>
+          <t>Reynosa</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>28032</t>
-        </is>
+      <c r="A13" s="1" t="n">
+        <v>28032</v>
       </c>
       <c r="B13" t="n">
         <v>0</v>
@@ -628,22 +612,22 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>32056</t>
+          <t>19026</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Zacatecas</t>
+          <t>Guadalupe</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>32056</t>
+          <t>28038</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -651,90 +635,84 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Zacatecas</t>
+          <t>Tampico</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>14039</t>
+          <t>32056</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Zacatecas</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>07034</t>
-        </is>
+      <c r="A17" s="1" t="n">
+        <v>32056</v>
       </c>
       <c r="B17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Frontera Comalapa</t>
+          <t>Zacatecas</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>11015</t>
-        </is>
+      <c r="A18" s="1" t="n">
+        <v>32056</v>
       </c>
       <c r="B18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Guanajuato</t>
+          <t>Zacatecas</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>25011</t>
+          <t>32056</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Guasave</t>
+          <t>Zacatecas</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>32017</t>
+          <t>26030</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Guadalupe</t>
+          <t>Hermosillo</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>16003</t>
-        </is>
+      <c r="A21" s="1" t="n">
+        <v>16003</v>
       </c>
       <c r="B21" t="n">
         <v>0</v>
@@ -746,24 +724,22 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>04009</t>
-        </is>
+      <c r="A22" s="1" t="n">
+        <v>11015</v>
       </c>
       <c r="B22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Escárcega</t>
+          <t>Guanajuato</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>20043</t>
+          <t>10007</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -771,29 +747,27 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Heroica Ciudad de Juchitán de Zaragoza</t>
+          <t>Gómez Palacio</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>05013</t>
-        </is>
+      <c r="A24" s="1" t="n">
+        <v>25011</v>
       </c>
       <c r="B24" t="n">
         <v>0</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Hidalgo</t>
+          <t>Guasave</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>07037</t>
+          <t>20043</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -801,119 +775,107 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
+          <t>Heroica Ciudad de Juchitán de Zaragoza</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="n">
+        <v>19026</v>
+      </c>
+      <c r="B26" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Guadalupe</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n">
+        <v>26030</v>
+      </c>
+      <c r="B27" t="n">
+        <v>1</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Hermosillo</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="n">
+        <v>7037</v>
+      </c>
+      <c r="B28" t="n">
+        <v>1</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
           <t>Huehuetán</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="1" t="inlineStr">
-        <is>
-          <t>27008</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>0</v>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Huimanguillo</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="1" t="inlineStr">
-        <is>
-          <t>07040</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>1</v>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Huixtla</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="1" t="inlineStr">
-        <is>
-          <t>11017</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>0</v>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Irapuato</t>
-        </is>
-      </c>
-    </row>
     <row r="29">
-      <c r="A29" s="1" t="inlineStr">
-        <is>
-          <t>15039</t>
-        </is>
+      <c r="A29" s="1" t="n">
+        <v>20043</v>
       </c>
       <c r="B29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Ixtapaluca</t>
+          <t>Heroica Ciudad de Juchitán de Zaragoza</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="inlineStr">
-        <is>
-          <t>09007</t>
-        </is>
+      <c r="A30" s="1" t="n">
+        <v>8035</v>
       </c>
       <c r="B30" t="n">
         <v>1</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Iztapalapa</t>
+          <t>Janos</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>08035</t>
+          <t>16052</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Janos</t>
+          <t>Lázaro Cárdenas</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="inlineStr">
-        <is>
-          <t>26030</t>
-        </is>
+      <c r="A32" s="1" t="n">
+        <v>11020</v>
       </c>
       <c r="B32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Hermosillo</t>
+          <t>León</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>09015</t>
+          <t>11020</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -921,14 +883,14 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Cuauhtémoc</t>
+          <t>León</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>25009</t>
+          <t>08037</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -936,74 +898,68 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Escuinapa</t>
+          <t>Juárez</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="inlineStr">
-        <is>
-          <t>07012</t>
-        </is>
+      <c r="A35" s="1" t="n">
+        <v>8037</v>
       </c>
       <c r="B35" t="n">
         <v>0</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Berriozábal</t>
+          <t>Juárez</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="inlineStr">
-        <is>
-          <t>30003</t>
-        </is>
+      <c r="A36" s="1" t="n">
+        <v>1005</v>
       </c>
       <c r="B36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Acayucan</t>
+          <t>Jesús María</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>05002</t>
+          <t>08035</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Acuña</t>
+          <t>Janos</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="inlineStr">
-        <is>
-          <t>01001</t>
-        </is>
+      <c r="A38" s="1" t="n">
+        <v>9007</v>
       </c>
       <c r="B38" t="n">
         <v>1</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Aguascalientes</t>
+          <t>Iztapalapa</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>25001</t>
+          <t>05013</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1011,44 +967,42 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Ahome</t>
+          <t>Hidalgo</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>15010</t>
+          <t>09007</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Apaxco</t>
+          <t>Iztapalapa</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="inlineStr">
-        <is>
-          <t>29002</t>
-        </is>
+      <c r="A41" s="1" t="n">
+        <v>15039</v>
       </c>
       <c r="B41" t="n">
         <v>0</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Apetatitlán de Antonio Carvajal</t>
+          <t>Ixtapaluca</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>19006</t>
+          <t>11017</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1056,74 +1010,70 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Apodaca</t>
+          <t>Irapuato</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>07009</t>
+          <t>07040</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Arriaga</t>
+          <t>Huixtla</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="inlineStr">
-        <is>
-          <t>15014</t>
-        </is>
+      <c r="A44" s="1" t="n">
+        <v>7040</v>
       </c>
       <c r="B44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Atlacomulco</t>
+          <t>Huixtla</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>23005</t>
+          <t>27008</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Benito Juárez</t>
+          <t>Huimanguillo</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="inlineStr">
-        <is>
-          <t>04002</t>
-        </is>
+      <c r="A46" s="1" t="n">
+        <v>14039</v>
       </c>
       <c r="B46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Campeche</t>
+          <t>Guadalajara</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>10005</t>
+          <t>32017</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1131,29 +1081,27 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Durango</t>
+          <t>Guadalupe</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="inlineStr">
-        <is>
-          <t>11007</t>
-        </is>
+      <c r="A48" s="1" t="n">
+        <v>25009</v>
       </c>
       <c r="B48" t="n">
         <v>0</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Celaya</t>
+          <t>Escuinapa</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>27004</t>
+          <t>14039</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1161,14 +1109,14 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Centro</t>
+          <t>Guadalajara</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>15025</t>
+          <t>11007</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1176,14 +1124,14 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Chalco</t>
+          <t>Celaya</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>07027</t>
+          <t>07012</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1191,74 +1139,68 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Chiapa de Corzo</t>
+          <t>Berriozábal</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>08019</t>
+          <t>23005</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Chihuahua</t>
+          <t>Benito Juárez</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="1" t="inlineStr">
-        <is>
-          <t>20014</t>
-        </is>
+      <c r="A53" s="1" t="n">
+        <v>23005</v>
       </c>
       <c r="B53" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Ciudad Ixtepec</t>
+          <t>Benito Juárez</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="1" t="inlineStr">
-        <is>
-          <t>30039</t>
-        </is>
+      <c r="A54" s="1" t="n">
+        <v>15014</v>
       </c>
       <c r="B54" t="n">
         <v>0</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Coatzacoalcos</t>
+          <t>Atlacomulco</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="inlineStr">
-        <is>
-          <t>07019</t>
-        </is>
+      <c r="A55" s="1" t="n">
+        <v>7009</v>
       </c>
       <c r="B55" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Comitán de Domínguez</t>
+          <t>Arriaga</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>08037</t>
+          <t>07009</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1266,14 +1208,14 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Juárez</t>
+          <t>Arriaga</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>25006</t>
+          <t>19006</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1281,119 +1223,109 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Culiacán</t>
+          <t>Apodaca</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="1" t="inlineStr">
-        <is>
-          <t>01005</t>
-        </is>
+      <c r="A58" s="1" t="n">
+        <v>29002</v>
       </c>
       <c r="B58" t="n">
         <v>0</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Jesús María</t>
+          <t>Apetatitlán de Antonio Carvajal</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="1" t="inlineStr">
-        <is>
-          <t>30108</t>
-        </is>
+      <c r="A59" s="1" t="n">
+        <v>15010</v>
       </c>
       <c r="B59" t="n">
         <v>0</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Minatitlán</t>
+          <t>Apaxco</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="1" t="inlineStr">
-        <is>
-          <t>11020</t>
-        </is>
+      <c r="A60" s="1" t="n">
+        <v>25001</v>
       </c>
       <c r="B60" t="n">
         <v>0</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>León</t>
+          <t>Ahome</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>15095</t>
+          <t>01001</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Tepotzotlán</t>
+          <t>Aguascalientes</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="1" t="inlineStr">
-        <is>
-          <t>24028</t>
-        </is>
+      <c r="A62" s="1" t="n">
+        <v>5002</v>
       </c>
       <c r="B62" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>San Luis Potosí</t>
+          <t>Acuña</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="1" t="inlineStr">
-        <is>
-          <t>11003</t>
-        </is>
+      <c r="A63" s="1" t="n">
+        <v>30003</v>
       </c>
       <c r="B63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>San Miguel de Allende</t>
+          <t>Acayucan</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>20327</t>
+          <t>30003</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>San Pedro Tapanatepec</t>
+          <t>Acayucan</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>20413</t>
+          <t>12001</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1401,104 +1333,92 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Santa María Huatulco</t>
+          <t>Acapulco de Juárez</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="1" t="inlineStr">
-        <is>
-          <t>20418</t>
-        </is>
+      <c r="A66" s="1" t="n">
+        <v>4002</v>
       </c>
       <c r="B66" t="n">
         <v>0</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Santa María Jalapa del Marqués</t>
+          <t>Campeche</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="1" t="inlineStr">
-        <is>
-          <t>07087</t>
-        </is>
+      <c r="A67" s="1" t="n">
+        <v>11007</v>
       </c>
       <c r="B67" t="n">
         <v>0</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Suchiate</t>
+          <t>Celaya</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="1" t="inlineStr">
-        <is>
-          <t>07089</t>
-        </is>
+      <c r="A68" s="1" t="n">
+        <v>7034</v>
       </c>
       <c r="B68" t="n">
         <v>1</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Tapachula</t>
+          <t>Frontera Comalapa</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="1" t="inlineStr">
-        <is>
-          <t>27017</t>
-        </is>
+      <c r="A69" s="1" t="n">
+        <v>27004</v>
       </c>
       <c r="B69" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Tenosique</t>
+          <t>Centro</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="1" t="inlineStr">
-        <is>
-          <t>18017</t>
-        </is>
+      <c r="A70" s="1" t="n">
+        <v>4009</v>
       </c>
       <c r="B70" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Tepic</t>
+          <t>Escárcega</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="1" t="inlineStr">
-        <is>
-          <t>02004</t>
-        </is>
+      <c r="A71" s="1" t="n">
+        <v>25012</v>
       </c>
       <c r="B71" t="n">
         <v>1</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Tijuana</t>
+          <t>Mazatlán</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>16052</t>
+          <t>10005</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1506,14 +1426,14 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Lázaro Cárdenas</t>
+          <t>Durango</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>15104</t>
+          <t>25006</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1521,29 +1441,27 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Tlalnepantla de Baz</t>
+          <t>Culiacán</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="1" t="inlineStr">
-        <is>
-          <t>29033</t>
-        </is>
+      <c r="A74" s="1" t="n">
+        <v>9015</v>
       </c>
       <c r="B74" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Tlaxcala</t>
+          <t>Cuauhtémoc</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>15106</t>
+          <t>09015</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1551,29 +1469,27 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Toluca</t>
+          <t>Cuauhtémoc</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="1" t="inlineStr">
-        <is>
-          <t>07097</t>
-        </is>
+      <c r="A76" s="1" t="n">
+        <v>7019</v>
       </c>
       <c r="B76" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Tonalá</t>
+          <t>Comitán de Domínguez</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>05035</t>
+          <t>07019</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1581,14 +1497,14 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Torreón</t>
+          <t>Comitán de Domínguez</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>07102</t>
+          <t>30039</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1596,29 +1512,27 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Tuxtla Chico</t>
+          <t>Coatzacoalcos</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="1" t="inlineStr">
-        <is>
-          <t>07101</t>
-        </is>
+      <c r="A79" s="1" t="n">
+        <v>20014</v>
       </c>
       <c r="B79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Tuxtla Gutiérrez</t>
+          <t>Ciudad Ixtepec</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>09017</t>
+          <t>20014</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1626,14 +1540,14 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Venustiano Carranza</t>
+          <t>Ciudad Ixtepec</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>28041</t>
+          <t>08019</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1641,44 +1555,42 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Victoria</t>
+          <t>Chihuahua</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>07078</t>
+          <t>07027</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>San Cristóbal de las Casas</t>
+          <t>Chiapa de Corzo</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="1" t="inlineStr">
-        <is>
-          <t>20083</t>
-        </is>
+      <c r="A83" s="1" t="n">
+        <v>15025</v>
       </c>
       <c r="B83" t="n">
         <v>0</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>San Agustín de las Juntas</t>
+          <t>Chalco</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>05030</t>
+          <t>27004</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1686,29 +1598,27 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Saltillo</t>
+          <t>Centro</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="1" t="inlineStr">
-        <is>
-          <t>20079</t>
-        </is>
+      <c r="A85" s="1" t="n">
+        <v>28022</v>
       </c>
       <c r="B85" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Salina Cruz</t>
+          <t>Matamoros</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>28022</t>
+          <t>16053</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1716,7 +1626,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Matamoros</t>
+          <t>Morelia</t>
         </is>
       </c>
     </row>
@@ -1736,69 +1646,63 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="1" t="inlineStr">
-        <is>
-          <t>15120</t>
-        </is>
+      <c r="A88" s="1" t="n">
+        <v>20418</v>
       </c>
       <c r="B88" t="n">
         <v>0</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Zumpango</t>
+          <t>Santa María Jalapa del Marqués</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="1" t="inlineStr">
-        <is>
-          <t>05018</t>
-        </is>
+      <c r="A89" s="1" t="n">
+        <v>18017</v>
       </c>
       <c r="B89" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Monclova</t>
+          <t>Tepic</t>
         </is>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="1" t="inlineStr">
-        <is>
-          <t>19039</t>
-        </is>
+      <c r="A90" s="1" t="n">
+        <v>27017</v>
       </c>
       <c r="B90" t="n">
         <v>0</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Monterrey</t>
+          <t>Tenosique</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>16053</t>
+          <t>27017</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Morelia</t>
+          <t>Tenosique</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>31050</t>
+          <t>07089</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1806,44 +1710,40 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Mérida</t>
+          <t>Tapachula</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="1" t="inlineStr">
-        <is>
-          <t>05022</t>
-        </is>
+      <c r="A93" s="1" t="n">
+        <v>7089</v>
       </c>
       <c r="B93" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Nava</t>
+          <t>Tapachula</t>
         </is>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="1" t="inlineStr">
-        <is>
-          <t>28027</t>
-        </is>
+      <c r="A94" s="1" t="n">
+        <v>7087</v>
       </c>
       <c r="B94" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Nuevo Laredo</t>
+          <t>Suchiate</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>30116</t>
+          <t>20418</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1851,29 +1751,27 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Oluta</t>
+          <t>Santa María Jalapa del Marqués</t>
         </is>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="1" t="inlineStr">
-        <is>
-          <t>23004</t>
-        </is>
+      <c r="A96" s="1" t="n">
+        <v>24028</v>
       </c>
       <c r="B96" t="n">
         <v>1</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Othón P. Blanco</t>
+          <t>San Luis Potosí</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>13048</t>
+          <t>20413</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1881,125 +1779,817 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Pachuca de Soto</t>
+          <t>Santa María Huatulco</t>
         </is>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="1" t="inlineStr">
-        <is>
-          <t>07065</t>
-        </is>
+      <c r="A98" s="1" t="n">
+        <v>20413</v>
       </c>
       <c r="B98" t="n">
         <v>1</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Palenque</t>
+          <t>Santa María Huatulco</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>05025</t>
+          <t>20327</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Piedras Negras</t>
+          <t>San Pedro Tapanatepec</t>
         </is>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="1" t="inlineStr">
-        <is>
-          <t>07069</t>
-        </is>
+      <c r="A100" s="1" t="n">
+        <v>20327</v>
       </c>
       <c r="B100" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Pijijiapan</t>
+          <t>San Pedro Tapanatepec</t>
         </is>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="1" t="inlineStr">
-        <is>
-          <t>21114</t>
-        </is>
+      <c r="A101" s="1" t="n">
+        <v>11003</v>
       </c>
       <c r="B101" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Puebla</t>
+          <t>San Miguel de Allende</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>22014</t>
+          <t>11003</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Querétaro</t>
+          <t>San Miguel de Allende</t>
         </is>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="1" t="inlineStr">
-        <is>
-          <t>05027</t>
-        </is>
+      <c r="A103" s="1" t="n">
+        <v>15095</v>
       </c>
       <c r="B103" t="n">
         <v>0</v>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Ramos Arizpe</t>
+          <t>Tepotzotlán</t>
         </is>
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="1" t="inlineStr">
-        <is>
-          <t>11027</t>
-        </is>
+      <c r="A104" s="1" t="n">
+        <v>2004</v>
       </c>
       <c r="B104" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Salamanca</t>
+          <t>Tijuana</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>12001</t>
+          <t>02004</t>
         </is>
       </c>
       <c r="B105" t="n">
         <v>1</v>
       </c>
       <c r="C105" t="inlineStr">
+        <is>
+          <t>Tijuana</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="1" t="n">
+        <v>15104</v>
+      </c>
+      <c r="B106" t="n">
+        <v>0</v>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Tlalnepantla de Baz</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="1" t="n">
+        <v>29033</v>
+      </c>
+      <c r="B107" t="n">
+        <v>1</v>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Tlaxcala</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="1" t="n">
+        <v>15106</v>
+      </c>
+      <c r="B108" t="n">
+        <v>0</v>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Toluca</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="1" t="inlineStr">
+        <is>
+          <t>15106</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>0</v>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Toluca</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="1" t="inlineStr">
+        <is>
+          <t>07097</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>0</v>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Tonalá</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="1" t="inlineStr">
+        <is>
+          <t>05035</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>1</v>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Torreón</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="1" t="n">
+        <v>5035</v>
+      </c>
+      <c r="B112" t="n">
+        <v>1</v>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Torreón</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="1" t="inlineStr">
+        <is>
+          <t>07102</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>0</v>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Tuxtla Chico</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="1" t="inlineStr">
+        <is>
+          <t>07101</t>
+        </is>
+      </c>
+      <c r="B114" t="n">
+        <v>1</v>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Tuxtla Gutiérrez</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="1" t="n">
+        <v>7101</v>
+      </c>
+      <c r="B115" t="n">
+        <v>1</v>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Tuxtla Gutiérrez</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="1" t="inlineStr">
+        <is>
+          <t>09017</t>
+        </is>
+      </c>
+      <c r="B116" t="n">
+        <v>0</v>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Venustiano Carranza</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="1" t="inlineStr">
+        <is>
+          <t>30193</t>
+        </is>
+      </c>
+      <c r="B117" t="n">
+        <v>1</v>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Veracruz</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="1" t="n">
+        <v>30193</v>
+      </c>
+      <c r="B118" t="n">
+        <v>0</v>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Veracruz</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="1" t="n">
+        <v>28041</v>
+      </c>
+      <c r="B119" t="n">
+        <v>0</v>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Victoria</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="1" t="inlineStr">
+        <is>
+          <t>24028</t>
+        </is>
+      </c>
+      <c r="B120" t="n">
+        <v>1</v>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>San Luis Potosí</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="1" t="n">
+        <v>7078</v>
+      </c>
+      <c r="B121" t="n">
+        <v>1</v>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>San Cristóbal de las Casas</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="1" t="inlineStr">
+        <is>
+          <t>30108</t>
+        </is>
+      </c>
+      <c r="B122" t="n">
+        <v>0</v>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Minatitlán</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="1" t="inlineStr">
+        <is>
+          <t>28027</t>
+        </is>
+      </c>
+      <c r="B123" t="n">
+        <v>1</v>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Nuevo Laredo</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="1" t="inlineStr">
+        <is>
+          <t>13048</t>
+        </is>
+      </c>
+      <c r="B124" t="n">
+        <v>1</v>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Pachuca de Soto</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="1" t="inlineStr">
+        <is>
+          <t>23004</t>
+        </is>
+      </c>
+      <c r="B125" t="n">
+        <v>1</v>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Othón P. Blanco</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="1" t="n">
+        <v>23004</v>
+      </c>
+      <c r="B126" t="n">
+        <v>1</v>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Othón P. Blanco</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="1" t="inlineStr">
+        <is>
+          <t>30116</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>0</v>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Oluta</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="1" t="inlineStr">
+        <is>
+          <t>20067</t>
+        </is>
+      </c>
+      <c r="B128" t="n">
+        <v>1</v>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Oaxaca de Juárez</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="1" t="n">
+        <v>28027</v>
+      </c>
+      <c r="B129" t="n">
+        <v>1</v>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Nuevo Laredo</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="1" t="inlineStr">
+        <is>
+          <t>05022</t>
+        </is>
+      </c>
+      <c r="B130" t="n">
+        <v>0</v>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Nava</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="1" t="inlineStr">
+        <is>
+          <t>07078</t>
+        </is>
+      </c>
+      <c r="B131" t="n">
+        <v>1</v>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>San Cristóbal de las Casas</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="1" t="n">
+        <v>31050</v>
+      </c>
+      <c r="B132" t="n">
+        <v>1</v>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Mérida</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="1" t="inlineStr">
+        <is>
+          <t>15120</t>
+        </is>
+      </c>
+      <c r="B133" t="n">
+        <v>0</v>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Zumpango</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="1" t="n">
+        <v>16053</v>
+      </c>
+      <c r="B134" t="n">
+        <v>1</v>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Morelia</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="1" t="inlineStr">
+        <is>
+          <t>19039</t>
+        </is>
+      </c>
+      <c r="B135" t="n">
+        <v>0</v>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Monterrey</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="1" t="inlineStr">
+        <is>
+          <t>05018</t>
+        </is>
+      </c>
+      <c r="B136" t="n">
+        <v>1</v>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Monclova</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="1" t="n">
+        <v>5018</v>
+      </c>
+      <c r="B137" t="n">
+        <v>1</v>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Monclova</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="1" t="n">
+        <v>13048</v>
+      </c>
+      <c r="B138" t="n">
+        <v>1</v>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Pachuca de Soto</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="1" t="inlineStr">
+        <is>
+          <t>07065</t>
+        </is>
+      </c>
+      <c r="B139" t="n">
+        <v>1</v>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Palenque</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="1" t="n">
+        <v>7065</v>
+      </c>
+      <c r="B140" t="n">
+        <v>1</v>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Palenque</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="1" t="inlineStr">
+        <is>
+          <t>05025</t>
+        </is>
+      </c>
+      <c r="B141" t="n">
+        <v>1</v>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Piedras Negras</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="1" t="n">
+        <v>5025</v>
+      </c>
+      <c r="B142" t="n">
+        <v>1</v>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Piedras Negras</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="1" t="n">
+        <v>7069</v>
+      </c>
+      <c r="B143" t="n">
+        <v>1</v>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Pijijiapan</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="1" t="inlineStr">
+        <is>
+          <t>07069</t>
+        </is>
+      </c>
+      <c r="B144" t="n">
+        <v>1</v>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Pijijiapan</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="1" t="inlineStr">
+        <is>
+          <t>21114</t>
+        </is>
+      </c>
+      <c r="B145" t="n">
+        <v>1</v>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Puebla</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="1" t="n">
+        <v>21114</v>
+      </c>
+      <c r="B146" t="n">
+        <v>1</v>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Puebla</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="1" t="n">
+        <v>22014</v>
+      </c>
+      <c r="B147" t="n">
+        <v>1</v>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Querétaro</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="1" t="inlineStr">
+        <is>
+          <t>22014</t>
+        </is>
+      </c>
+      <c r="B148" t="n">
+        <v>1</v>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Querétaro</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="1" t="inlineStr">
+        <is>
+          <t>05027</t>
+        </is>
+      </c>
+      <c r="B149" t="n">
+        <v>0</v>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Ramos Arizpe</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="1" t="n">
+        <v>11027</v>
+      </c>
+      <c r="B150" t="n">
+        <v>0</v>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Salamanca</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="1" t="n">
+        <v>20079</v>
+      </c>
+      <c r="B151" t="n">
+        <v>0</v>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Salina Cruz</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="1" t="inlineStr">
+        <is>
+          <t>05030</t>
+        </is>
+      </c>
+      <c r="B152" t="n">
+        <v>1</v>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Saltillo</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="1" t="n">
+        <v>5030</v>
+      </c>
+      <c r="B153" t="n">
+        <v>1</v>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Saltillo</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="1" t="n">
+        <v>20083</v>
+      </c>
+      <c r="B154" t="n">
+        <v>0</v>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>San Agustín de las Juntas</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="1" t="n">
+        <v>12001</v>
+      </c>
+      <c r="B155" t="n">
+        <v>1</v>
+      </c>
+      <c r="C155" t="inlineStr">
         <is>
           <t>Acapulco de Juárez</t>
         </is>

</xml_diff>